<commit_message>
Fix rekap export logic and add job logs trait
Corrects several issues in the SPKL rekap export and enhances the LaporanUpload model.

- Fix duration calculation by correcting the diffInMinutes argument order, ensuring negative durations are handled and small durations are skipped.
- Collect pegawai names into a map and write Nama Pegawai into the spreadsheet when the header exists.
- Change default column mapping (NIP Lama default to B, Nama Pegawai default to A) and write NIP values explicitly as strings to preserve formatting/leading zeros.
- Minor formatting/flow cleanups in the loop.
- Add HasJobLogs trait to App\Models\Simple\LaporanUpload for job logging support.
- Update the Excel template (binary) used for the rekap export.

These changes fix incorrect hour calculations, include employee names in exports, and ensure NIP values are preserved in the generated spreadsheet.
</commit_message>
<xml_diff>
--- a/public/document/template_rekap utk uang.xlsx
+++ b/public/document/template_rekap utk uang.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rifqind\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\xampp\htdocs\singkat\public\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{175F1512-4657-49AC-9F3E-9E5DA5CB7F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6203DA79-8DD0-41F1-84FE-0A8712AF585E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8D25137E-22AB-4F2F-8C7D-B798D3086879}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>NIP Lama</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>HL16</t>
+  </si>
+  <si>
+    <t>Nama Pegawai</t>
   </si>
 </sst>
 </file>
@@ -169,9 +172,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,95 +511,101 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D4FBC0C-A289-4C36-B824-9B1CC430D4CC}">
-  <dimension ref="A1:AC1"/>
+  <dimension ref="A1:AD1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="8.88671875" style="2"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>